<commit_message>
Polish flashcards portfolio project
</commit_message>
<xml_diff>
--- a/vocab.xlsx
+++ b/vocab.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="181">
   <si>
     <t>set</t>
   </si>
@@ -22,7 +22,7 @@
     <t>en</t>
   </si>
   <si>
-    <t>🔵Word 第 1 組</t>
+    <t>🔵Word 01</t>
   </si>
   <si>
     <t>文档</t>
@@ -31,30 +31,45 @@
     <t>Document</t>
   </si>
   <si>
+    <t>run</t>
+  </si>
+  <si>
     <t>字体</t>
   </si>
   <si>
     <t>Font</t>
   </si>
   <si>
+    <t>cd path/to/flashcards</t>
+  </si>
+  <si>
     <t>字号</t>
   </si>
   <si>
     <t>Size</t>
   </si>
   <si>
+    <t>npm init -y</t>
+  </si>
+  <si>
     <t>加粗</t>
   </si>
   <si>
     <t>Bold</t>
   </si>
   <si>
+    <t>npm i xlsx</t>
+  </si>
+  <si>
     <t>倾斜</t>
   </si>
   <si>
     <t>Italic</t>
   </si>
   <si>
+    <t>🔵Word 02</t>
+  </si>
+  <si>
     <t>下划线</t>
   </si>
   <si>
@@ -85,7 +100,7 @@
     <t>Align Left</t>
   </si>
   <si>
-    <t>🔵Word 第 2 組</t>
+    <t>🔵Word 03</t>
   </si>
   <si>
     <t>居中</t>
@@ -118,6 +133,9 @@
     <t>Indent</t>
   </si>
   <si>
+    <t>🔵Word 04</t>
+  </si>
+  <si>
     <t>项目符号</t>
   </si>
   <si>
@@ -148,7 +166,7 @@
     <t>Orientation</t>
   </si>
   <si>
-    <t>🔵Word 第 3 組</t>
+    <t>🔵Word 05</t>
   </si>
   <si>
     <t>纵向</t>
@@ -181,6 +199,9 @@
     <t>Footer</t>
   </si>
   <si>
+    <t>🔵Word 06</t>
+  </si>
+  <si>
     <t>分隔符</t>
   </si>
   <si>
@@ -211,7 +232,7 @@
     <t>Column</t>
   </si>
   <si>
-    <t>🔵Word 第 4 組</t>
+    <t>🔵Word 07</t>
   </si>
   <si>
     <t>单元格</t>
@@ -244,6 +265,9 @@
     <t>Shape</t>
   </si>
   <si>
+    <t>🔵Word 08</t>
+  </si>
+  <si>
     <t>文本框</t>
   </si>
   <si>
@@ -274,7 +298,7 @@
     <t>Crop</t>
   </si>
   <si>
-    <t>🔵Word 第 5 組</t>
+    <t>🔵Word 09</t>
   </si>
   <si>
     <t>剪切</t>
@@ -307,6 +331,9 @@
     <t>Find</t>
   </si>
   <si>
+    <t>🔵Word 10</t>
+  </si>
+  <si>
     <t>替换</t>
   </si>
   <si>
@@ -337,7 +364,7 @@
     <t>Proofing</t>
   </si>
   <si>
-    <t>🔵Word 第 6 組</t>
+    <t>🔵Word 11</t>
   </si>
   <si>
     <t>样式</t>
@@ -370,6 +397,9 @@
     <t>Mail merge</t>
   </si>
   <si>
+    <t>🔵Word 12</t>
+  </si>
+  <si>
     <t>信封</t>
   </si>
   <si>
@@ -400,7 +430,7 @@
     <t>Review</t>
   </si>
   <si>
-    <t>🔵Word 第 7 組</t>
+    <t>🔵Word 13</t>
   </si>
   <si>
     <t>接受</t>
@@ -433,6 +463,9 @@
     <t>Copies</t>
   </si>
   <si>
+    <t>🔵Word 14</t>
+  </si>
+  <si>
     <t>页数</t>
   </si>
   <si>
@@ -451,7 +484,7 @@
     <t>Ruler</t>
   </si>
   <si>
-    <t>🔵Word 第 8 組</t>
+    <t>🔵Word 15</t>
   </si>
   <si>
     <t>功能区</t>
@@ -482,6 +515,9 @@
   </si>
   <si>
     <t>Save</t>
+  </si>
+  <si>
+    <t>🔵Word 16</t>
   </si>
   <si>
     <t>另存为</t>
@@ -580,7 +616,9 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
@@ -825,16 +863,28 @@
       <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
+      <c r="D2" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="D3" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -842,10 +892,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -853,10 +906,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -864,846 +920,846 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>